<commit_message>
re-organize and update the inventory sorting
</commit_message>
<xml_diff>
--- a/separated_by_section/Accessible_Transportation.xlsx
+++ b/separated_by_section/Accessible_Transportation.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P194"/>
+  <dimension ref="A1:P248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -429,11 +429,11 @@
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
     <col width="39" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="31" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
@@ -13743,6 +13743,3710 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" s="1" t="n">
+        <v>571133</v>
+      </c>
+      <c r="B195" s="1" t="inlineStr">
+        <is>
+          <t>Accessibility at the Canadian Transportation Agency</t>
+        </is>
+      </c>
+      <c r="C195" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/accessibility-at-canadian-transportation-agency</t>
+        </is>
+      </c>
+      <c r="D195" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/laccessibilite-a-loffice-des-transports-canada</t>
+        </is>
+      </c>
+      <c r="E195" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, January 6, 2026</t>
+        </is>
+      </c>
+      <c r="F195" s="1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G195" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H195" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I195" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J195" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K195" s="1" t="inlineStr"/>
+      <c r="L195" s="1" t="n">
+        <v>729</v>
+      </c>
+      <c r="M195" s="1" t="n">
+        <v>980</v>
+      </c>
+      <c r="N195" s="1" t="n">
+        <v>831</v>
+      </c>
+      <c r="O195" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P195" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="1" t="n">
+        <v>570665</v>
+      </c>
+      <c r="B196" s="1" t="inlineStr">
+        <is>
+          <t>Compensation for accessibility-related complaints</t>
+        </is>
+      </c>
+      <c r="C196" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/compensation-accessibility-related-complaints</t>
+        </is>
+      </c>
+      <c r="D196" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/indemnite-pour-plaintes-relatives-a-laccessibilite</t>
+        </is>
+      </c>
+      <c r="E196" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, March 3, 2026</t>
+        </is>
+      </c>
+      <c r="F196" s="1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G196" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H196" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I196" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J196" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K196" s="1" t="inlineStr"/>
+      <c r="L196" s="1" t="n">
+        <v>336</v>
+      </c>
+      <c r="M196" s="1" t="n">
+        <v>489</v>
+      </c>
+      <c r="N196" s="1" t="n">
+        <v>493</v>
+      </c>
+      <c r="O196" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P196" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="1" t="n">
+        <v>93852</v>
+      </c>
+      <c r="B197" s="1" t="inlineStr">
+        <is>
+          <t>Contact an enforcement officer</t>
+        </is>
+      </c>
+      <c r="C197" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/regional-enforcement-officers</t>
+        </is>
+      </c>
+      <c r="D197" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/agents-verbalisateurs-regionaux</t>
+        </is>
+      </c>
+      <c r="E197" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, May 14, 2025</t>
+        </is>
+      </c>
+      <c r="F197" s="1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G197" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H197" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I197" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J197" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K197" s="1" t="inlineStr"/>
+      <c r="L197" s="1" t="n">
+        <v>2477</v>
+      </c>
+      <c r="M197" s="1" t="n">
+        <v>3123</v>
+      </c>
+      <c r="N197" s="1" t="n">
+        <v>3021</v>
+      </c>
+      <c r="O197" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P197" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="1" t="n">
+        <v>569291</v>
+      </c>
+      <c r="B198" s="1" t="inlineStr">
+        <is>
+          <t>NOTICE: Opportunity to apply for appointment by the Governor in Council to a roster from which Temporary Members of the Canadian Transportation Agency are selected</t>
+        </is>
+      </c>
+      <c r="C198" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/notice-opportunity-apply-appointment-governor-council-a-roster-which-temporary-members</t>
+        </is>
+      </c>
+      <c r="D198" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/avis-possibilite-postuler-pour-une-nomination-par-gouverneur-conseil-pour-etre-inscrit-a-une</t>
+        </is>
+      </c>
+      <c r="E198" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, May 5, 2020</t>
+        </is>
+      </c>
+      <c r="F198" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G198" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H198" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I198" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J198" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K198" s="1" t="inlineStr"/>
+      <c r="L198" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="M198" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="N198" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="O198" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P198" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="1" t="n">
+        <v>568981</v>
+      </c>
+      <c r="B199" s="1" t="inlineStr">
+        <is>
+          <t>Canadian Transportation Agency launches consultation on Phase II of its Accessible Transportation for Persons with Disabilities Regulations</t>
+        </is>
+      </c>
+      <c r="C199" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/canadian-transportation-agency-launches-consultation-phase-ii-its-accessible-transportation</t>
+        </is>
+      </c>
+      <c r="D199" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/loffice-des-transports-canada-lance-des-consultations-sur-phase-ii-son-reglement-sur</t>
+        </is>
+      </c>
+      <c r="E199" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, December 3, 2019</t>
+        </is>
+      </c>
+      <c r="F199" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G199" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H199" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I199" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J199" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K199" s="1" t="inlineStr"/>
+      <c r="L199" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="M199" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="N199" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="O199" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P199" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="1" t="n">
+        <v>568957</v>
+      </c>
+      <c r="B200" s="1" t="inlineStr">
+        <is>
+          <t>Notice of Oral Hearing: Application by Timothy Rose against Air Canada</t>
+        </is>
+      </c>
+      <c r="C200" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/notice-oral-hearing-application-timothy-rose-against-air-canada</t>
+        </is>
+      </c>
+      <c r="D200" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/avis-daudience-publique-demande-deposee-par-timothy-rose-contre-air-canada</t>
+        </is>
+      </c>
+      <c r="E200" s="1" t="inlineStr">
+        <is>
+          <t>Friday, November 22, 2019</t>
+        </is>
+      </c>
+      <c r="F200" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G200" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H200" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I200" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J200" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K200" s="1" t="inlineStr"/>
+      <c r="L200" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="M200" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="N200" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="O200" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P200" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="1" t="n">
+        <v>568835</v>
+      </c>
+      <c r="B201" s="1" t="inlineStr">
+        <is>
+          <t>Canadian Transportation Agency issues International Working Group's recommendations on mobility aids and air travel</t>
+        </is>
+      </c>
+      <c r="C201" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/canadian-transportation-agency-issues-international-working-groups-recommendations-mobility</t>
+        </is>
+      </c>
+      <c r="D201" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/loffice-des-transports-canada-publie-recommandations-groupe-travail-international-sur-aides</t>
+        </is>
+      </c>
+      <c r="E201" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, September 10, 2019</t>
+        </is>
+      </c>
+      <c r="F201" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G201" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H201" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I201" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J201" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K201" s="1" t="inlineStr"/>
+      <c r="L201" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="M201" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="N201" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="O201" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P201" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="1" t="n">
+        <v>573257</v>
+      </c>
+      <c r="B202" s="1" t="inlineStr">
+        <is>
+          <t>Departmental results report 2024–25: Response to parliamentary committees and external audits</t>
+        </is>
+      </c>
+      <c r="C202" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/publication/departmental-results-report-2024-25-response-parliamentary-committees-and-external</t>
+        </is>
+      </c>
+      <c r="D202" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/publication/rapport-sur-resultats-ministeriels-2024-2025-reponse-aux-comites-parlementaires-et-aux</t>
+        </is>
+      </c>
+      <c r="E202" s="1" t="inlineStr">
+        <is>
+          <t>Friday, November 7, 2025</t>
+        </is>
+      </c>
+      <c r="F202" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G202" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H202" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I202" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J202" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K202" s="1" t="inlineStr"/>
+      <c r="L202" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="M202" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="N202" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="O202" s="1" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="P202" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="1" t="n">
+        <v>573026</v>
+      </c>
+      <c r="B203" s="1" t="inlineStr">
+        <is>
+          <t>Reporting obligations under the Fighting Against Forced Labour and Child Labour in Supply Chains Act 2024-2025</t>
+        </is>
+      </c>
+      <c r="C203" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/publication/reporting-obligations-under-fighting-against-forced-labour-and-child-labour-supply-2024-2025</t>
+        </is>
+      </c>
+      <c r="D203" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/publication/obligations-faire-rapport-vertu-loi-sur-lutte-contre-travail-force-et-travail-des-2024-2025</t>
+        </is>
+      </c>
+      <c r="E203" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, May 29, 2025</t>
+        </is>
+      </c>
+      <c r="F203" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G203" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H203" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I203" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J203" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K203" s="1" t="inlineStr"/>
+      <c r="L203" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="M203" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="N203" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="O203" s="1" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="P203" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="1" t="n">
+        <v>573222</v>
+      </c>
+      <c r="B204" s="1" t="inlineStr">
+        <is>
+          <t>Megantic - Vanity URL</t>
+        </is>
+      </c>
+      <c r="C204" s="1" t="inlineStr"/>
+      <c r="D204" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra</t>
+        </is>
+      </c>
+      <c r="E204" s="1" t="inlineStr">
+        <is>
+          <t>Friday, October 24, 2025</t>
+        </is>
+      </c>
+      <c r="F204" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G204" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H204" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I204" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J204" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K204" s="1" t="inlineStr">
+        <is>
+          <t>Missing EN; Possible orphan — confirm</t>
+        </is>
+      </c>
+      <c r="L204" s="1" t="inlineStr"/>
+      <c r="M204" s="1" t="inlineStr"/>
+      <c r="N204" s="1" t="inlineStr"/>
+      <c r="O204" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P204" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="1" t="n">
+        <v>571136</v>
+      </c>
+      <c r="B205" s="1" t="inlineStr">
+        <is>
+          <t>Accessibility feedback process at the Canadian Transportation Agency</t>
+        </is>
+      </c>
+      <c r="C205" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/accessibility-feedback-process-at-canadian-transportation-agency</t>
+        </is>
+      </c>
+      <c r="D205" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/processus-retroaction-sur-laccessibilite-a-loffice-des-transports-canada</t>
+        </is>
+      </c>
+      <c r="E205" s="1" t="inlineStr">
+        <is>
+          <t>Friday, May 5, 2023</t>
+        </is>
+      </c>
+      <c r="F205" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G205" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H205" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I205" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J205" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K205" s="1" t="inlineStr"/>
+      <c r="L205" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="M205" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="N205" s="1" t="n">
+        <v>69</v>
+      </c>
+      <c r="O205" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P205" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="1" t="n">
+        <v>571039</v>
+      </c>
+      <c r="B206" s="1" t="inlineStr">
+        <is>
+          <t>Members Code of Conduct</t>
+        </is>
+      </c>
+      <c r="C206" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/members-code-conduct</t>
+        </is>
+      </c>
+      <c r="D206" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/code-conduite-des-membres</t>
+        </is>
+      </c>
+      <c r="E206" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, November 24, 2022</t>
+        </is>
+      </c>
+      <c r="F206" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G206" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H206" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I206" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J206" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K206" s="1" t="inlineStr"/>
+      <c r="L206" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="M206" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="N206" s="1" t="n">
+        <v>78</v>
+      </c>
+      <c r="O206" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P206" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="1" t="n">
+        <v>570434</v>
+      </c>
+      <c r="B207" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation Planning and Reporting Regulations</t>
+        </is>
+      </c>
+      <c r="C207" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/accessible-transportation-planning-and-reporting-regulations</t>
+        </is>
+      </c>
+      <c r="D207" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/reglement-sur-letablissement-des-plans-et-des-rapports-matiere-transports-accessibles</t>
+        </is>
+      </c>
+      <c r="E207" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, December 22, 2021</t>
+        </is>
+      </c>
+      <c r="F207" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G207" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H207" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I207" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J207" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K207" s="1" t="inlineStr"/>
+      <c r="L207" s="1" t="n">
+        <v>679</v>
+      </c>
+      <c r="M207" s="1" t="n">
+        <v>1218</v>
+      </c>
+      <c r="N207" s="1" t="n">
+        <v>1099</v>
+      </c>
+      <c r="O207" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P207" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="1" t="n">
+        <v>570012</v>
+      </c>
+      <c r="B208" s="1" t="inlineStr">
+        <is>
+          <t>Transcripts from working group meetings on the Temporary Exemption Requests from the Accessible Transportation for Persons with Disabilities Regulations</t>
+        </is>
+      </c>
+      <c r="C208" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/transcripts-working-group-meetings-temporary-exemption-requests-accessible-transportation-persons</t>
+        </is>
+      </c>
+      <c r="D208" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/transcriptions-des-reunions-groupe-travail-sur-demandes-dexemption-temporaire-lapplication-reglement</t>
+        </is>
+      </c>
+      <c r="E208" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, May 5, 2021</t>
+        </is>
+      </c>
+      <c r="F208" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G208" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H208" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I208" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J208" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K208" s="1" t="inlineStr"/>
+      <c r="L208" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="M208" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="N208" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="O208" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P208" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="1" t="n">
+        <v>569912</v>
+      </c>
+      <c r="B209" s="1" t="inlineStr">
+        <is>
+          <t>Request for Conditional Exemptions from the Accessible Transportation for Persons with Disabilities Regulations</t>
+        </is>
+      </c>
+      <c r="C209" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/request-conditional-exemptions-accessible-transportation-persons-disabilities-regulations</t>
+        </is>
+      </c>
+      <c r="D209" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/demande-dexemptions-conditionnelles-lapplication-reglement-sur-transports-accessibles-aux-personnes</t>
+        </is>
+      </c>
+      <c r="E209" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, March 3, 2021</t>
+        </is>
+      </c>
+      <c r="F209" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G209" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H209" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I209" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J209" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K209" s="1" t="inlineStr"/>
+      <c r="L209" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="M209" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="N209" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="O209" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P209" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="1" t="n">
+        <v>569880</v>
+      </c>
+      <c r="B210" s="1" t="inlineStr">
+        <is>
+          <t>American Sign Language version : Summary of the Proposed Accessible Transportation Planning and Reporting Regulations</t>
+        </is>
+      </c>
+      <c r="C210" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/american-sign-language-version-summary-proposed-accessible-transportation-planning-and-reporting</t>
+        </is>
+      </c>
+      <c r="D210" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/version-langue-des-signes-quebecoise-resume-version-proposee-reglement-sur-letablissement-des-plans</t>
+        </is>
+      </c>
+      <c r="E210" s="1" t="inlineStr">
+        <is>
+          <t>Saturday, February 13, 2021</t>
+        </is>
+      </c>
+      <c r="F210" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G210" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H210" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I210" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J210" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K210" s="1" t="inlineStr"/>
+      <c r="L210" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="M210" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="N210" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="O210" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P210" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="1" t="n">
+        <v>569515</v>
+      </c>
+      <c r="B211" s="1" t="inlineStr">
+        <is>
+          <t>International Civil Aviation Organization</t>
+        </is>
+      </c>
+      <c r="C211" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/international-civil-aviation-organization</t>
+        </is>
+      </c>
+      <c r="D211" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/organisation-laviation-civile-internationale</t>
+        </is>
+      </c>
+      <c r="E211" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, August 26, 2020</t>
+        </is>
+      </c>
+      <c r="F211" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G211" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H211" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I211" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J211" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K211" s="1" t="inlineStr"/>
+      <c r="L211" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="M211" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="N211" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="O211" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P211" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="1" t="n">
+        <v>281685</v>
+      </c>
+      <c r="B212" s="1" t="inlineStr">
+        <is>
+          <t>Acts and regulations</t>
+        </is>
+      </c>
+      <c r="C212" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/acts-and-regulations</t>
+        </is>
+      </c>
+      <c r="D212" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/lois-et-reglements-accueil</t>
+        </is>
+      </c>
+      <c r="E212" s="1" t="inlineStr">
+        <is>
+          <t>Monday, July 8, 2019</t>
+        </is>
+      </c>
+      <c r="F212" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G212" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H212" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I212" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J212" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K212" s="1" t="inlineStr"/>
+      <c r="L212" s="1" t="n">
+        <v>1896</v>
+      </c>
+      <c r="M212" s="1" t="n">
+        <v>2454</v>
+      </c>
+      <c r="N212" s="1" t="n">
+        <v>2284</v>
+      </c>
+      <c r="O212" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P212" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="1" t="n">
+        <v>93574</v>
+      </c>
+      <c r="B213" s="1" t="inlineStr">
+        <is>
+          <t>Careers at the Canadian Transportation Agency</t>
+        </is>
+      </c>
+      <c r="C213" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/careers</t>
+        </is>
+      </c>
+      <c r="D213" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/carrieres</t>
+        </is>
+      </c>
+      <c r="E213" s="1" t="inlineStr">
+        <is>
+          <t>Friday, March 21, 2025</t>
+        </is>
+      </c>
+      <c r="F213" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G213" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H213" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I213" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J213" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K213" s="1" t="inlineStr"/>
+      <c r="L213" s="1" t="n">
+        <v>3005</v>
+      </c>
+      <c r="M213" s="1" t="n">
+        <v>3670</v>
+      </c>
+      <c r="N213" s="1" t="n">
+        <v>3367</v>
+      </c>
+      <c r="O213" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P213" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="1" t="n">
+        <v>572487</v>
+      </c>
+      <c r="B214" s="1" t="inlineStr">
+        <is>
+          <t>National AccessAbility Week – Message from the Chair</t>
+        </is>
+      </c>
+      <c r="C214" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/national-accessability-week-message-chair-1</t>
+        </is>
+      </c>
+      <c r="D214" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/semaine-nationale-laccessibilite-message-presidente-0</t>
+        </is>
+      </c>
+      <c r="E214" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, May 28, 2024</t>
+        </is>
+      </c>
+      <c r="F214" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G214" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H214" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I214" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J214" s="1" t="inlineStr">
+        <is>
+          <t>Unsure</t>
+        </is>
+      </c>
+      <c r="K214" s="1" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+      <c r="L214" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="M214" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="N214" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="O214" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P214" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="1" t="n">
+        <v>572294</v>
+      </c>
+      <c r="B215" s="1" t="inlineStr">
+        <is>
+          <t>Canadian Transportation Agency recognized as one of the National Capital Region's top employers for 2024</t>
+        </is>
+      </c>
+      <c r="C215" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/cta-recognized-one-ncr-top-employers-2024</t>
+        </is>
+      </c>
+      <c r="D215" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/otc-reconnu-lun-meilleurs-employers-region-capital-2024</t>
+        </is>
+      </c>
+      <c r="E215" s="1" t="inlineStr">
+        <is>
+          <t>Friday, February 9, 2024</t>
+        </is>
+      </c>
+      <c r="F215" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G215" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H215" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I215" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J215" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K215" s="1" t="inlineStr"/>
+      <c r="L215" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="M215" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="N215" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="O215" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P215" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="1" t="n">
+        <v>572494</v>
+      </c>
+      <c r="B216" s="1" t="inlineStr">
+        <is>
+          <t>Reporting obligations under the Fighting Against Forced Labour and Child Labour in Supply Chains Act 2023-2024</t>
+        </is>
+      </c>
+      <c r="C216" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/publication/reporting-obligations-under-fighting-against-forced-labour-and-child-labour-supply</t>
+        </is>
+      </c>
+      <c r="D216" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/publication/obligations-faire-rapport-vertu-loi-sur-lutte-contre-travail-force-et-travail-des</t>
+        </is>
+      </c>
+      <c r="E216" s="1" t="inlineStr">
+        <is>
+          <t>Friday, May 31, 2024</t>
+        </is>
+      </c>
+      <c r="F216" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G216" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H216" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I216" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J216" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K216" s="1" t="inlineStr"/>
+      <c r="L216" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="M216" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="N216" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="O216" s="1" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="P216" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="1" t="n">
+        <v>572799</v>
+      </c>
+      <c r="B217" s="1" t="inlineStr">
+        <is>
+          <t>Joint ICAO/ACI/IATA Symposium on Accessibility in International Civil Aviation - December 2, 2024</t>
+        </is>
+      </c>
+      <c r="C217" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/joint-icaoaciiata-symposium-accessibility-international-civil-aviation-december-2-2024</t>
+        </is>
+      </c>
+      <c r="D217" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/contenu/symposium-conjoint-loaci-laci-et-liata-sur-laccessibilite-aviation-civile-internationale-2</t>
+        </is>
+      </c>
+      <c r="E217" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, December 3, 2024</t>
+        </is>
+      </c>
+      <c r="F217" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G217" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H217" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I217" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J217" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K217" s="1" t="inlineStr"/>
+      <c r="L217" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="M217" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="N217" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="O217" s="1" t="inlineStr">
+        <is>
+          <t>Speeches</t>
+        </is>
+      </c>
+      <c r="P217" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="1" t="n">
+        <v>572821</v>
+      </c>
+      <c r="B218" s="1" t="inlineStr">
+        <is>
+          <t>Accessibility progress reports</t>
+        </is>
+      </c>
+      <c r="C218" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/accessibility-progress-reports</t>
+        </is>
+      </c>
+      <c r="D218" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/rapports-detape-sur-laccessibilite</t>
+        </is>
+      </c>
+      <c r="E218" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, December 18, 2024</t>
+        </is>
+      </c>
+      <c r="F218" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G218" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H218" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I218" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J218" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K218" s="1" t="inlineStr"/>
+      <c r="L218" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="M218" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="N218" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="O218" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P218" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="1" t="n">
+        <v>572753</v>
+      </c>
+      <c r="B219" s="1" t="inlineStr">
+        <is>
+          <t>Departmental results report 2023–24: Response to parliamentary committees and external audits</t>
+        </is>
+      </c>
+      <c r="C219" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/departmental-results-report-2023-24-response-parliamentary-committees-and-external-audits</t>
+        </is>
+      </c>
+      <c r="D219" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/rapport-sur-resultats-ministeriels-2023-2024-reponse-aux-comites-parlementaires-et-aux-audits</t>
+        </is>
+      </c>
+      <c r="E219" s="1" t="inlineStr">
+        <is>
+          <t>Friday, November 8, 2024</t>
+        </is>
+      </c>
+      <c r="F219" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G219" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H219" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I219" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J219" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K219" s="1" t="inlineStr"/>
+      <c r="L219" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="M219" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="N219" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="O219" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P219" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="1" t="n">
+        <v>572326</v>
+      </c>
+      <c r="B220" s="1" t="inlineStr">
+        <is>
+          <t>Canadian Transportation Agency’s 2024-2025 Departmental plan at a glance</t>
+        </is>
+      </c>
+      <c r="C220" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/canadian-transportation-agencys-2024-2025-departmental-plan-at-a-glance</t>
+        </is>
+      </c>
+      <c r="D220" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/apercu-plan-ministeriel-2024-2025-loffice-des-transports-canada</t>
+        </is>
+      </c>
+      <c r="E220" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, February 29, 2024</t>
+        </is>
+      </c>
+      <c r="F220" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G220" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H220" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I220" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J220" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K220" s="1" t="inlineStr"/>
+      <c r="L220" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="M220" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="N220" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="O220" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P220" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="1" t="n">
+        <v>567919</v>
+      </c>
+      <c r="B221" s="1" t="inlineStr">
+        <is>
+          <t>Local Media Advisory ‒ The Canadian Transportation Agency's air passenger protection in-person consultations come to Toronto</t>
+        </is>
+      </c>
+      <c r="C221" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/local-media-advisory-canadian-transportation-agencys-air-passenger-protection-person</t>
+        </is>
+      </c>
+      <c r="D221" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/avis-aux-medias-locaux-consultations-personne-loffice-des-transports-canada-sur-protection</t>
+        </is>
+      </c>
+      <c r="E221" s="1" t="inlineStr">
+        <is>
+          <t>Monday, June 11, 2018</t>
+        </is>
+      </c>
+      <c r="F221" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G221" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H221" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I221" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J221" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K221" s="1" t="inlineStr"/>
+      <c r="L221" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="M221" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="N221" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="O221" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P221" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="1" t="n">
+        <v>567918</v>
+      </c>
+      <c r="B222" s="1" t="inlineStr">
+        <is>
+          <t>The Canadian Transportation Agency launches in-person air passenger protection consultations</t>
+        </is>
+      </c>
+      <c r="C222" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/canadian-transportation-agency-launches-person-air-passenger-protection-consultations</t>
+        </is>
+      </c>
+      <c r="D222" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/loffice-des-transports-canada-lance-des-consultations-personne-sur-protection-des-passagers</t>
+        </is>
+      </c>
+      <c r="E222" s="1" t="inlineStr">
+        <is>
+          <t>Monday, June 11, 2018</t>
+        </is>
+      </c>
+      <c r="F222" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G222" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H222" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I222" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J222" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K222" s="1" t="inlineStr"/>
+      <c r="L222" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="M222" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="N222" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="O222" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P222" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="1" t="n">
+        <v>565455</v>
+      </c>
+      <c r="B223" s="1" t="inlineStr">
+        <is>
+          <t>Canadian Transportation Agency launches consultation on accessible transportation as Phase 1 of its Regulatory Modernization Initiative</t>
+        </is>
+      </c>
+      <c r="C223" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/canadian-transportation-agency-launches-consultation-accessible-transportation-phase-1-its</t>
+        </is>
+      </c>
+      <c r="D223" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/loffice-des-transports-canada-lance-une-consultation-sur-transports-accessibles-dans-cadre</t>
+        </is>
+      </c>
+      <c r="E223" s="1" t="inlineStr">
+        <is>
+          <t>Monday, June 6, 2016</t>
+        </is>
+      </c>
+      <c r="F223" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G223" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H223" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I223" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J223" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K223" s="1" t="inlineStr"/>
+      <c r="L223" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="M223" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="N223" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="O223" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P223" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="1" t="n">
+        <v>572118</v>
+      </c>
+      <c r="B224" s="1" t="inlineStr">
+        <is>
+          <t>Departmental Results Report 2022-2023: Response to parliamentary committees and external audits</t>
+        </is>
+      </c>
+      <c r="C224" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/departmental-results-report-2022-2023-response-parliamentary-committees-and-external-audits</t>
+        </is>
+      </c>
+      <c r="D224" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/rapport-sur-resultats-ministeriels-2022-2023-reponse-aux-comites-parlementaires-et-aux-audits</t>
+        </is>
+      </c>
+      <c r="E224" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, November 9, 2023</t>
+        </is>
+      </c>
+      <c r="F224" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G224" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H224" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I224" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J224" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K224" s="1" t="inlineStr"/>
+      <c r="L224" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="M224" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="N224" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="O224" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P224" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="1" t="n">
+        <v>562767</v>
+      </c>
+      <c r="B225" s="1" t="inlineStr">
+        <is>
+          <t>FAQs: Personnel Training for the Assistance of Persons with Disabilities Regulations</t>
+        </is>
+      </c>
+      <c r="C225" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/faqs-personnel-training-assistance-persons-with-disabilities-regulations</t>
+        </is>
+      </c>
+      <c r="D225" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/faq-reglement-sur-formation-personnel-matiere-daide-aux-personnes-ayant-une-deficience</t>
+        </is>
+      </c>
+      <c r="E225" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, December 23, 2014</t>
+        </is>
+      </c>
+      <c r="F225" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G225" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H225" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I225" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J225" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K225" s="1" t="inlineStr"/>
+      <c r="L225" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="M225" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="N225" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="O225" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P225" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="1" t="n">
+        <v>281790</v>
+      </c>
+      <c r="B226" s="1" t="inlineStr">
+        <is>
+          <t>Code of Values and Ethics for the Canadian Transportation Agency</t>
+        </is>
+      </c>
+      <c r="C226" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/publication/code-values-and-ethics-canadian-transportation-agency</t>
+        </is>
+      </c>
+      <c r="D226" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/publication/code-valeurs-et-dethique-loffice-des-transports-canada</t>
+        </is>
+      </c>
+      <c r="E226" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, October 6, 2015</t>
+        </is>
+      </c>
+      <c r="F226" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G226" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H226" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I226" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J226" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K226" s="1" t="inlineStr"/>
+      <c r="L226" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="M226" s="1" t="n">
+        <v>121</v>
+      </c>
+      <c r="N226" s="1" t="n">
+        <v>121</v>
+      </c>
+      <c r="O226" s="1" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="P226" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="1" t="n">
+        <v>567131</v>
+      </c>
+      <c r="B227" s="1" t="inlineStr">
+        <is>
+          <t>Interview with Scott Streiner, President and CEO, Canadian Transportation Agency, at the International Transportation Forum, 2017 Summit (from May 31 to June 2, 2017)</t>
+        </is>
+      </c>
+      <c r="C227" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/interview-scott-streiner-president-and-ceo-canadian-transportation-agency-at-international</t>
+        </is>
+      </c>
+      <c r="D227" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/contenu/entrevue-avec-scott-streiner-president-et-premier-dirigeant-office-des-transports-canada-au</t>
+        </is>
+      </c>
+      <c r="E227" s="1" t="inlineStr">
+        <is>
+          <t>Monday, June 19, 2017</t>
+        </is>
+      </c>
+      <c r="F227" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G227" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H227" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I227" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J227" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K227" s="1" t="inlineStr"/>
+      <c r="L227" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="M227" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="N227" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="O227" s="1" t="inlineStr">
+        <is>
+          <t>Speeches</t>
+        </is>
+      </c>
+      <c r="P227" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="1" t="n">
+        <v>571130</v>
+      </c>
+      <c r="B228" s="1" t="inlineStr">
+        <is>
+          <t>Accessibility feedback form</t>
+        </is>
+      </c>
+      <c r="C228" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/accessibility-feedback-form</t>
+        </is>
+      </c>
+      <c r="D228" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/formulaire-retroaction-sur-laccessibilite</t>
+        </is>
+      </c>
+      <c r="E228" s="1" t="inlineStr"/>
+      <c r="F228" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G228" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H228" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I228" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J228" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K228" s="1" t="inlineStr"/>
+      <c r="L228" s="1" t="n">
+        <v>82</v>
+      </c>
+      <c r="M228" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="N228" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="O228" s="1" t="inlineStr">
+        <is>
+          <t>Webform</t>
+        </is>
+      </c>
+      <c r="P228" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="1" t="n">
+        <v>570433</v>
+      </c>
+      <c r="B229" s="1" t="inlineStr">
+        <is>
+          <t>The Accessible Transportation Planning and Reporting Regulations are now finalized</t>
+        </is>
+      </c>
+      <c r="C229" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/accessible-transportation-planning-and-reporting-regulations-are-now-finalized</t>
+        </is>
+      </c>
+      <c r="D229" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/reglement-sur-letablissement-des-plans-et-des-rapports-matiere-transports-accessibles-est</t>
+        </is>
+      </c>
+      <c r="E229" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, December 22, 2021</t>
+        </is>
+      </c>
+      <c r="F229" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G229" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H229" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I229" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J229" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K229" s="1" t="inlineStr"/>
+      <c r="L229" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="M229" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="N229" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="O229" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P229" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="1" t="n">
+        <v>570398</v>
+      </c>
+      <c r="B230" s="1" t="inlineStr">
+        <is>
+          <t>International Day of Persons with Disabilities 2021</t>
+        </is>
+      </c>
+      <c r="C230" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/international-day-persons-disabilities-2021</t>
+        </is>
+      </c>
+      <c r="D230" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/journee-internationale-des-personnes-situation-handicap-2021</t>
+        </is>
+      </c>
+      <c r="E230" s="1" t="inlineStr">
+        <is>
+          <t>Friday, December 3, 2021</t>
+        </is>
+      </c>
+      <c r="F230" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G230" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H230" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I230" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J230" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K230" s="1" t="inlineStr"/>
+      <c r="L230" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="M230" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="N230" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="O230" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P230" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="1" t="n">
+        <v>569392</v>
+      </c>
+      <c r="B231" s="1" t="inlineStr">
+        <is>
+          <t>New Accessible Transportation for Persons with Disabilities Regulations now in force</t>
+        </is>
+      </c>
+      <c r="C231" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/new-accessible-transportation-persons-disabilities-regulations-now-force</t>
+        </is>
+      </c>
+      <c r="D231" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/entree-vigueur-nouveau-reglement-sur-transports-accessibles-aux-personnes-handicapees</t>
+        </is>
+      </c>
+      <c r="E231" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, June 25, 2020</t>
+        </is>
+      </c>
+      <c r="F231" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G231" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H231" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I231" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J231" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K231" s="1" t="inlineStr"/>
+      <c r="L231" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="M231" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="N231" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="O231" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P231" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="1" t="n">
+        <v>568748</v>
+      </c>
+      <c r="B232" s="1" t="inlineStr">
+        <is>
+          <t>Notice of Oral Hearing: Application by Rosalie Finlay against Sunwing Airlines Inc. (Sunwing)</t>
+        </is>
+      </c>
+      <c r="C232" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/notice-oral-hearing-application-rosalie-finlay-against-sunwing-airlines-inc-sunwing</t>
+        </is>
+      </c>
+      <c r="D232" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/avis-daudience-demande-deposee-par-rosalie-finlay-contre-sunwing-airlines-inc-sunwing</t>
+        </is>
+      </c>
+      <c r="E232" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, July 11, 2019</t>
+        </is>
+      </c>
+      <c r="F232" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G232" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H232" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I232" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J232" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K232" s="1" t="inlineStr"/>
+      <c r="L232" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="M232" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="N232" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="O232" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P232" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="1" t="n">
+        <v>568221</v>
+      </c>
+      <c r="B233" s="1" t="inlineStr">
+        <is>
+          <t>Remarks from Chair and CEO, Scott Streiner, to the Standing Committee on Human Resources, Skills and Social Development and the Status of Persons with Disabilities</t>
+        </is>
+      </c>
+      <c r="C233" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/remarks-chair-and-ceo-scott-streiner-standing-committee-human-resources-skills-and-social-0</t>
+        </is>
+      </c>
+      <c r="D233" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/discours-president-et-premier-dirigeant-scott-streiner-a-lintention-comite-permanent-des</t>
+        </is>
+      </c>
+      <c r="E233" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, October 23, 2018</t>
+        </is>
+      </c>
+      <c r="F233" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G233" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H233" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I233" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J233" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K233" s="1" t="inlineStr"/>
+      <c r="L233" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="M233" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="N233" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="O233" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P233" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="1" t="n">
+        <v>569835</v>
+      </c>
+      <c r="B234" s="1" t="inlineStr">
+        <is>
+          <t>Temporary exemption requests from transportation service providers and submitted comments</t>
+        </is>
+      </c>
+      <c r="C234" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/temporary-exemption-requests-transportation-service-providers-and-submitted-comments</t>
+        </is>
+      </c>
+      <c r="D234" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/demandes-dexemption-temporaire-par-des-fournisseurs-services-transport-et-commentaires-soumis</t>
+        </is>
+      </c>
+      <c r="E234" s="1" t="inlineStr">
+        <is>
+          <t>Monday, January 18, 2021</t>
+        </is>
+      </c>
+      <c r="F234" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G234" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H234" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I234" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J234" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K234" s="1" t="inlineStr"/>
+      <c r="L234" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="M234" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="N234" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="O234" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P234" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="1" t="n">
+        <v>569389</v>
+      </c>
+      <c r="B235" s="1" t="inlineStr">
+        <is>
+          <t>Accessible transportation complaints help line</t>
+        </is>
+      </c>
+      <c r="C235" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/accessible-transportation-complaints-help-line</t>
+        </is>
+      </c>
+      <c r="D235" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/ligne-daide-relative-aux-plaintes-reliees-au-transport-accessible</t>
+        </is>
+      </c>
+      <c r="E235" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, June 23, 2020</t>
+        </is>
+      </c>
+      <c r="F235" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G235" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H235" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I235" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J235" s="1" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="K235" s="1" t="inlineStr"/>
+      <c r="L235" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M235" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="N235" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O235" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P235" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="1" t="n">
+        <v>569667</v>
+      </c>
+      <c r="B236" s="1" t="inlineStr">
+        <is>
+          <t>Chair and CEO Keynote Address to the IATA Global Accessibility Symposium – October 27, 2020</t>
+        </is>
+      </c>
+      <c r="C236" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/chair-and-ceo-keynote-address-iata-global-accessibility-symposium-october-27-2020</t>
+        </is>
+      </c>
+      <c r="D236" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/discours-president-et-premier-dirigeant-lors-symposium-mondial-liata-sur-laccessibilite-27</t>
+        </is>
+      </c>
+      <c r="E236" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, November 4, 2020</t>
+        </is>
+      </c>
+      <c r="F236" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G236" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H236" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I236" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J236" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K236" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L236" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="M236" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="N236" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="O236" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P236" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="1" t="n">
+        <v>569666</v>
+      </c>
+      <c r="B237" s="1" t="inlineStr">
+        <is>
+          <t>Agency releases its 2019-2020 Annual Report</t>
+        </is>
+      </c>
+      <c r="C237" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/agency-releases-its-2019-2020-annual-report</t>
+        </is>
+      </c>
+      <c r="D237" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/loffice-publie-son-rapport-annuel-2019-2020</t>
+        </is>
+      </c>
+      <c r="E237" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, November 4, 2020</t>
+        </is>
+      </c>
+      <c r="F237" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G237" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H237" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I237" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J237" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K237" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L237" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="M237" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="N237" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O237" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P237" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="1" t="n">
+        <v>568311</v>
+      </c>
+      <c r="B238" s="1" t="inlineStr">
+        <is>
+          <t>Statement by Chair and CEO Scott Streiner on International Day of Persons with Disabilities</t>
+        </is>
+      </c>
+      <c r="C238" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/statement-chair-and-ceo-scott-streiner-international-day-persons-with-disabilities</t>
+        </is>
+      </c>
+      <c r="D238" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/content/declaration-president-et-premier-dirigeant-scott-streiner-a-loccasion-journee-internationale</t>
+        </is>
+      </c>
+      <c r="E238" s="1" t="inlineStr">
+        <is>
+          <t>Monday, December 3, 2018</t>
+        </is>
+      </c>
+      <c r="F238" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G238" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H238" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I238" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J238" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K238" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L238" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="M238" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="N238" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="O238" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="P238" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="1" t="n">
+        <v>569740</v>
+      </c>
+      <c r="B239" s="1" t="inlineStr">
+        <is>
+          <t>Opening remarks from CTA Chair and CEO, Scott Streiner, to the Standing Committee on Transport, Infrastructure and Communities - December 1, 2020</t>
+        </is>
+      </c>
+      <c r="C239" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/opening-remarks-cta-chair-and-ceo-scott-streiner-standing-committee-transport-infrastructure</t>
+        </is>
+      </c>
+      <c r="D239" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/contenu/allocution-douverture-president-et-premier-dirigeant-scott-streiner-a-lintention-comite</t>
+        </is>
+      </c>
+      <c r="E239" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, December 3, 2020</t>
+        </is>
+      </c>
+      <c r="F239" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G239" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H239" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I239" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J239" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K239" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L239" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="M239" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="N239" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="O239" s="1" t="inlineStr">
+        <is>
+          <t>Speeches</t>
+        </is>
+      </c>
+      <c r="P239" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="1" t="n">
+        <v>569058</v>
+      </c>
+      <c r="B240" s="1" t="inlineStr">
+        <is>
+          <t>Audio version: Phase II – Consultation on ATPDR (General summary)</t>
+        </is>
+      </c>
+      <c r="C240" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/audio-version-phase-ii-consultation-atpdr-general-summary</t>
+        </is>
+      </c>
+      <c r="D240" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/version-audio-phase-ii-consultations-publiques-rtaph-resume-general</t>
+        </is>
+      </c>
+      <c r="E240" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, January 16, 2020</t>
+        </is>
+      </c>
+      <c r="F240" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G240" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H240" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I240" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J240" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K240" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L240" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="M240" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="N240" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="O240" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P240" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="1" t="n">
+        <v>568788</v>
+      </c>
+      <c r="B241" s="1" t="inlineStr">
+        <is>
+          <t>Highlights of one-person-one-fare policy decision</t>
+        </is>
+      </c>
+      <c r="C241" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/highlights-one-person-one-fare-policy-decision</t>
+        </is>
+      </c>
+      <c r="D241" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/points-saillants-decision-concernant-politique-une-personne-un-tarif</t>
+        </is>
+      </c>
+      <c r="E241" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, August 6, 2019</t>
+        </is>
+      </c>
+      <c r="F241" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G241" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H241" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I241" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J241" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K241" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L241" s="1" t="n">
+        <v>328</v>
+      </c>
+      <c r="M241" s="1" t="n">
+        <v>430</v>
+      </c>
+      <c r="N241" s="1" t="n">
+        <v>444</v>
+      </c>
+      <c r="O241" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P241" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="1" t="n">
+        <v>566855</v>
+      </c>
+      <c r="B242" s="1" t="inlineStr">
+        <is>
+          <t>Regulatory Modernization Initiative</t>
+        </is>
+      </c>
+      <c r="C242" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/regulatory-modernization-initiative</t>
+        </is>
+      </c>
+      <c r="D242" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/initiative-modernisation-reglementation</t>
+        </is>
+      </c>
+      <c r="E242" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, July 30, 2019</t>
+        </is>
+      </c>
+      <c r="F242" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G242" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H242" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I242" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J242" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K242" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L242" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="M242" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="N242" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="O242" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P242" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="1" t="n">
+        <v>568499</v>
+      </c>
+      <c r="B243" s="1" t="inlineStr">
+        <is>
+          <t>Chair and CEO Scott Streiner Announces Proposed Accessible Transportation for Persons with Disabilities Regulations on March 11, 2019</t>
+        </is>
+      </c>
+      <c r="C243" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/chair-and-ceo-scott-streiner-announces-proposed-accessible-transportation-persons-disabilities-regulations-march-11-2019</t>
+        </is>
+      </c>
+      <c r="D243" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/contenu/president-premier-dirigeant-Scott-Streiner-projet-reglement-transports-accessibles-personnes-handicapees-11-mars-2019</t>
+        </is>
+      </c>
+      <c r="E243" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday, March 12, 2019</t>
+        </is>
+      </c>
+      <c r="F243" s="1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G243" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H243" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I243" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J243" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K243" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L243" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="M243" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="N243" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="O243" s="1" t="inlineStr">
+        <is>
+          <t>Speeches</t>
+        </is>
+      </c>
+      <c r="P243" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="1" t="n">
+        <v>568682</v>
+      </c>
+      <c r="B244" s="1" t="inlineStr">
+        <is>
+          <t>Bill C-81 - The Accessible Canada Act</t>
+        </is>
+      </c>
+      <c r="C244" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/bill-c-81-accessible-canada-act</t>
+        </is>
+      </c>
+      <c r="D244" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/projet-loi-c-81-loi-canadienne-sur-laccessibilite</t>
+        </is>
+      </c>
+      <c r="E244" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, August 14, 2019</t>
+        </is>
+      </c>
+      <c r="F244" s="1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G244" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H244" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I244" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J244" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K244" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L244" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="M244" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="N244" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="O244" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P244" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="1" t="n">
+        <v>568560</v>
+      </c>
+      <c r="B245" s="1" t="inlineStr">
+        <is>
+          <t>2019-2020 Departmental Plan: Gender-based analysis plus</t>
+        </is>
+      </c>
+      <c r="C245" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/2019-2020-departmental-plan-gender-based-analysis-plus</t>
+        </is>
+      </c>
+      <c r="D245" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/plan-ministeriel-2019-2020-analyse-comparative-entre-sexes-plus</t>
+        </is>
+      </c>
+      <c r="E245" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, April 10, 2019</t>
+        </is>
+      </c>
+      <c r="F245" s="1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G245" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H245" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I245" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J245" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K245" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L245" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="M245" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="N245" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="O245" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P245" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="1" t="n">
+        <v>567783</v>
+      </c>
+      <c r="B246" s="1" t="inlineStr">
+        <is>
+          <t>Cleared for take-off: Regulatory reform and Canada's aviation sector</t>
+        </is>
+      </c>
+      <c r="C246" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/content/cleared-take-regulatory-reform-and-canadas-aviation-sector</t>
+        </is>
+      </c>
+      <c r="D246" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/contenu/autorise-a-decoller-reforme-reglementation-et-secteur-laviation-au-canada</t>
+        </is>
+      </c>
+      <c r="E246" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday, April 25, 2018</t>
+        </is>
+      </c>
+      <c r="F246" s="1" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G246" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H246" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I246" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J246" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K246" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L246" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="M246" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="N246" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="O246" s="1" t="inlineStr">
+        <is>
+          <t>Speeches</t>
+        </is>
+      </c>
+      <c r="P246" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="1" t="n">
+        <v>566237</v>
+      </c>
+      <c r="B247" s="1" t="inlineStr">
+        <is>
+          <t>Use of Social Media</t>
+        </is>
+      </c>
+      <c r="C247" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/eng/use-social-media</t>
+        </is>
+      </c>
+      <c r="D247" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/utilisation-des-medias-sociaux</t>
+        </is>
+      </c>
+      <c r="E247" s="1" t="inlineStr">
+        <is>
+          <t>Thursday, March 29, 2018</t>
+        </is>
+      </c>
+      <c r="F247" s="1" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G247" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H247" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I247" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J247" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K247" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated</t>
+        </is>
+      </c>
+      <c r="L247" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="M247" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="N247" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="O247" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P247" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="1" t="n">
+        <v>196423</v>
+      </c>
+      <c r="B248" s="1" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="C248" s="1" t="inlineStr"/>
+      <c r="D248" s="1" t="inlineStr">
+        <is>
+          <t>https://otc-cta.gc.ca/fra/news-0</t>
+        </is>
+      </c>
+      <c r="E248" s="1" t="inlineStr"/>
+      <c r="F248" s="1" t="n">
+        <v>2017</v>
+      </c>
+      <c r="G248" s="1" t="inlineStr">
+        <is>
+          <t>About / Contact / Corporate</t>
+        </is>
+      </c>
+      <c r="H248" s="1" t="inlineStr">
+        <is>
+          <t>Accessible Transportation</t>
+        </is>
+      </c>
+      <c r="I248" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J248" s="1" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K248" s="1" t="inlineStr">
+        <is>
+          <t>Possibly outdated; Missing EN; Possible orphan — confirm</t>
+        </is>
+      </c>
+      <c r="L248" s="1" t="inlineStr"/>
+      <c r="M248" s="1" t="inlineStr"/>
+      <c r="N248" s="1" t="inlineStr"/>
+      <c r="O248" s="1" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="P248" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>